<commit_message>
update centres csv data
</commit_message>
<xml_diff>
--- a/public/files/csv/centres.xlsx
+++ b/public/files/csv/centres.xlsx
@@ -1,28 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="26626"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\selection\public\files\csv\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\sigta\public\files\csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{709FA1B5-504D-42E8-BD6F-279541817558}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
     <sheet name="Feuil2" sheetId="2" r:id="rId2"/>
     <sheet name="Feuil3" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="48" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="60">
   <si>
     <t>centre</t>
   </si>
@@ -36,12 +35,6 @@
     <t>total</t>
   </si>
   <si>
-    <t>1°CFA/1°CRFI</t>
-  </si>
-  <si>
-    <t>2°CFA/2°CRFI</t>
-  </si>
-  <si>
     <t>EL HAJEB</t>
   </si>
   <si>
@@ -57,9 +50,6 @@
     <t>GUERCIF</t>
   </si>
   <si>
-    <t>A.BLINDEE</t>
-  </si>
-  <si>
     <t>2°BAFRA</t>
   </si>
   <si>
@@ -105,9 +95,6 @@
     <t>MARINE ROYALE</t>
   </si>
   <si>
-    <t>CISS</t>
-  </si>
-  <si>
     <t>TEMARA</t>
   </si>
   <si>
@@ -117,9 +104,6 @@
     <t>4°CFA</t>
   </si>
   <si>
-    <t>EM/ZS</t>
-  </si>
-  <si>
     <t>TANTAN</t>
   </si>
   <si>
@@ -135,19 +119,94 @@
     <t>6°CFA</t>
   </si>
   <si>
-    <t>ARM</t>
-  </si>
-  <si>
     <t>3°BUREAU</t>
   </si>
   <si>
     <t>3°CFA</t>
+  </si>
+  <si>
+    <t>1°CFA</t>
+  </si>
+  <si>
+    <t>2°CFA</t>
+  </si>
+  <si>
+    <t>BLINDEE</t>
+  </si>
+  <si>
+    <t>1°GEC</t>
+  </si>
+  <si>
+    <t>CAVALERIE</t>
+  </si>
+  <si>
+    <t>ERSS</t>
+  </si>
+  <si>
+    <t>1°CRFI</t>
+  </si>
+  <si>
+    <t>2°CRFI</t>
+  </si>
+  <si>
+    <t>7°GAR</t>
+  </si>
+  <si>
+    <t>1°BN</t>
+  </si>
+  <si>
+    <t>CASABLANCA</t>
+  </si>
+  <si>
+    <t>5°BMI</t>
+  </si>
+  <si>
+    <t>KHOURIBGA</t>
+  </si>
+  <si>
+    <t>12°RRC</t>
+  </si>
+  <si>
+    <t>MISSOUR</t>
+  </si>
+  <si>
+    <t>23°GAR</t>
+  </si>
+  <si>
+    <t>MIDELT</t>
+  </si>
+  <si>
+    <t>1°BG</t>
+  </si>
+  <si>
+    <t>MADIOUNA</t>
+  </si>
+  <si>
+    <t>GENIE</t>
+  </si>
+  <si>
+    <t>1GT</t>
+  </si>
+  <si>
+    <t>AIN HARROUDA</t>
+  </si>
+  <si>
+    <t>ATLOG</t>
+  </si>
+  <si>
+    <t>13°BRIMOTO</t>
+  </si>
+  <si>
+    <t>BOUARFA</t>
+  </si>
+  <si>
+    <t>BNI OUKIL</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -211,12 +270,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="1" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -235,9 +295,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Thème Office">
   <a:themeElements>
-    <a:clrScheme name="Office 2007 - 2010">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -275,9 +335,9 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2007 - 2010">
+    <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -312,7 +372,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -347,7 +407,7 @@
         <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2007 - 2010">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -520,8 +580,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.7109375" bestFit="1" customWidth="1"/>
@@ -529,7 +589,7 @@
     <col min="3" max="3" width="21.140625" customWidth="1"/>
     <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="13.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.25">
@@ -540,10 +600,10 @@
         <v>1</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>2</v>
@@ -554,292 +614,492 @@
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>6</v>
-      </c>
       <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D2" s="1">
-        <v>400</v>
-      </c>
-      <c r="E2" s="1">
-        <v>2600</v>
-      </c>
-      <c r="F2" s="1">
-        <v>3000</v>
+        <v>32</v>
+      </c>
+      <c r="D2" s="3">
+        <v>350</v>
+      </c>
+      <c r="E2" s="3">
+        <v>900</v>
+      </c>
+      <c r="F2">
+        <v>1250</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D3" s="1">
-        <v>350</v>
-      </c>
-      <c r="E3" s="1">
-        <v>2750</v>
-      </c>
-      <c r="F3" s="1">
-        <v>3100</v>
+        <v>32</v>
+      </c>
+      <c r="D3" s="3">
+        <v>300</v>
+      </c>
+      <c r="E3" s="3">
+        <v>1400</v>
+      </c>
+      <c r="F3">
+        <v>1700</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D4" s="1">
-        <v>0</v>
-      </c>
-      <c r="E4" s="1">
-        <v>2000</v>
-      </c>
-      <c r="F4" s="1">
-        <v>2000</v>
+        <v>32</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3">
+        <v>1850</v>
+      </c>
+      <c r="F4">
+        <v>1850</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0</v>
-      </c>
-      <c r="E5" s="1">
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3">
         <v>4000</v>
       </c>
-      <c r="F5" s="1">
+      <c r="F5">
         <v>4000</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0</v>
-      </c>
-      <c r="E6" s="1">
-        <v>2000</v>
-      </c>
-      <c r="F6" s="1">
-        <v>2000</v>
+        <v>32</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3">
+        <v>1850</v>
+      </c>
+      <c r="F6">
+        <v>1850</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0</v>
-      </c>
-      <c r="E7" s="1">
-        <v>2000</v>
-      </c>
-      <c r="F7" s="1">
-        <v>2000</v>
+        <v>32</v>
+      </c>
+      <c r="D7" s="3">
+        <v>0</v>
+      </c>
+      <c r="E7" s="3">
+        <v>1850</v>
+      </c>
+      <c r="F7">
+        <v>1850</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="1">
-        <v>500</v>
-      </c>
-      <c r="E8" s="1">
-        <v>1500</v>
-      </c>
-      <c r="F8" s="1">
-        <v>2000</v>
+        <v>32</v>
+      </c>
+      <c r="D8" s="3">
+        <v>400</v>
+      </c>
+      <c r="E8" s="3">
+        <v>1150</v>
+      </c>
+      <c r="F8">
+        <v>1550</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0</v>
-      </c>
-      <c r="E9" s="1">
-        <v>400</v>
-      </c>
-      <c r="F9" s="1">
-        <v>400</v>
+        <v>32</v>
+      </c>
+      <c r="D9" s="3">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3">
+        <v>450</v>
+      </c>
+      <c r="F9">
+        <v>450</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>16</v>
+        <v>6</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0</v>
-      </c>
-      <c r="E10" s="1">
-        <v>300</v>
-      </c>
-      <c r="F10" s="1">
-        <v>300</v>
+        <v>32</v>
+      </c>
+      <c r="D10" s="3">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3">
+        <v>1100</v>
+      </c>
+      <c r="F10">
+        <v>1100</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>17</v>
+        <v>43</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>18</v>
+        <v>44</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D11" s="1">
-        <v>0</v>
-      </c>
-      <c r="E11" s="1">
-        <v>400</v>
-      </c>
-      <c r="F11" s="1">
-        <v>400</v>
+        <v>23</v>
+      </c>
+      <c r="D11" s="3">
+        <v>200</v>
+      </c>
+      <c r="E11" s="3">
+        <v>500</v>
+      </c>
+      <c r="F11">
+        <v>700</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>20</v>
+        <v>46</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D12" s="1">
-        <v>0</v>
-      </c>
-      <c r="E12" s="1">
-        <v>200</v>
-      </c>
-      <c r="F12" s="1">
-        <v>200</v>
+        <v>36</v>
+      </c>
+      <c r="D12" s="3">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3">
+        <v>400</v>
+      </c>
+      <c r="F12">
+        <v>400</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>37</v>
+        <v>47</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>14</v>
+        <v>48</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="D13" s="1">
-        <v>0</v>
-      </c>
-      <c r="E13" s="1">
-        <v>50</v>
-      </c>
-      <c r="F13" s="1">
-        <v>50</v>
+        <v>36</v>
+      </c>
+      <c r="D13" s="3">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3">
+        <v>200</v>
+      </c>
+      <c r="F13">
+        <v>200</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>21</v>
+        <v>49</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D14" s="1">
-        <v>200</v>
-      </c>
-      <c r="E14" s="1">
-        <v>0</v>
-      </c>
-      <c r="F14" s="1">
-        <v>200</v>
+        <v>20</v>
+      </c>
+      <c r="D14" s="3">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3">
+        <v>150</v>
+      </c>
+      <c r="F14">
+        <v>150</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>27</v>
+        <v>51</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>28</v>
+        <v>52</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="1">
+        <v>53</v>
+      </c>
+      <c r="D15" s="3">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3">
+        <v>200</v>
+      </c>
+      <c r="F15">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="D16" s="3">
+        <v>0</v>
+      </c>
+      <c r="E16" s="3">
+        <v>200</v>
+      </c>
+      <c r="F16">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="D17" s="3">
+        <v>0</v>
+      </c>
+      <c r="E17" s="3">
+        <v>200</v>
+      </c>
+      <c r="F17">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="3">
+        <v>0</v>
+      </c>
+      <c r="E18" s="3">
+        <v>300</v>
+      </c>
+      <c r="F18">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A19" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D19" s="3">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3">
+        <v>400</v>
+      </c>
+      <c r="F19">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A20" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D20" s="3">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3">
+        <v>300</v>
+      </c>
+      <c r="F20">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="3">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3">
+        <v>400</v>
+      </c>
+      <c r="F21">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A22" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D22" s="3">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3">
+        <v>200</v>
+      </c>
+      <c r="F22">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A23" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D23" s="3">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3">
+        <v>200</v>
+      </c>
+      <c r="F23">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A24" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D24" s="3">
+        <v>200</v>
+      </c>
+      <c r="E24" s="3">
+        <v>0</v>
+      </c>
+      <c r="F24">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A25" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D25" s="3">
         <v>350</v>
       </c>
-      <c r="E15" s="1">
-        <v>0</v>
-      </c>
-      <c r="F15" s="1">
+      <c r="E25" s="3">
+        <v>0</v>
+      </c>
+      <c r="F25">
         <v>350</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -848,7 +1108,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>